<commit_message>
fixando os países sede
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="88">
   <si>
     <t>TIME</t>
   </si>
@@ -143,16 +143,10 @@
     <t>POL</t>
   </si>
   <si>
-    <t>SWE</t>
-  </si>
-  <si>
     <t>WAL</t>
   </si>
   <si>
-    <t>HUN</t>
-  </si>
-  <si>
-    <t>SER</t>
+    <t>SRB</t>
   </si>
   <si>
     <t>DRC</t>
@@ -164,6 +158,9 @@
     <t>PAN</t>
   </si>
   <si>
+    <t>GRE</t>
+  </si>
+  <si>
     <t>VEN</t>
   </si>
   <si>
@@ -176,6 +173,9 @@
     <t>SAF</t>
   </si>
   <si>
+    <t>IRL</t>
+  </si>
+  <si>
     <t>TUN</t>
   </si>
   <si>
@@ -209,73 +209,70 @@
     <t>OMA</t>
   </si>
   <si>
+    <t>SYR</t>
+  </si>
+  <si>
+    <t>NZE</t>
+  </si>
+  <si>
+    <t>OFC</t>
+  </si>
+  <si>
+    <t>CPV</t>
+  </si>
+  <si>
+    <t>NCL</t>
+  </si>
+  <si>
+    <t>MKD</t>
+  </si>
+  <si>
+    <t>GEO</t>
+  </si>
+  <si>
     <t>CUW</t>
   </si>
   <si>
-    <t>SYR</t>
-  </si>
-  <si>
-    <t>NZE</t>
-  </si>
-  <si>
-    <t>OFC</t>
-  </si>
-  <si>
-    <t>SCO</t>
-  </si>
-  <si>
-    <t>GRE</t>
+    <t>FEDERAÇÃO</t>
+  </si>
+  <si>
+    <t>6+1</t>
+  </si>
+  <si>
+    <t>6+2</t>
+  </si>
+  <si>
+    <t>8+1</t>
+  </si>
+  <si>
+    <t>9+1</t>
+  </si>
+  <si>
+    <t>1+1</t>
+  </si>
+  <si>
+    <t>REPESCAGEM</t>
+  </si>
+  <si>
+    <t>6(2)</t>
+  </si>
+  <si>
+    <t>8(4)</t>
+  </si>
+  <si>
+    <t>ANG</t>
+  </si>
+  <si>
+    <t>PER</t>
+  </si>
+  <si>
+    <t>CHN</t>
   </si>
   <si>
     <t>CHI</t>
   </si>
   <si>
-    <t>CPV</t>
-  </si>
-  <si>
-    <t>FEDERAÇÃO</t>
-  </si>
-  <si>
-    <t>20+2</t>
-  </si>
-  <si>
-    <t>6+1</t>
-  </si>
-  <si>
-    <t>7+1</t>
-  </si>
-  <si>
-    <t>6+2</t>
-  </si>
-  <si>
-    <t>8+1</t>
-  </si>
-  <si>
-    <t>12+1</t>
-  </si>
-  <si>
-    <t>9+1</t>
-  </si>
-  <si>
-    <t>1+1</t>
-  </si>
-  <si>
-    <t>REPESCAGEM</t>
-  </si>
-  <si>
-    <t>6(2)</t>
-  </si>
-  <si>
-    <t>8(4)</t>
-  </si>
-  <si>
-    <t>NCA</t>
-  </si>
-  <si>
-    <t>HAI</t>
-  </si>
-  <si>
-    <t>CHN</t>
+    <t>SOL</t>
   </si>
   <si>
     <t>GHA</t>
@@ -367,7 +364,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -393,6 +390,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -1042,7 +1042,7 @@
         <v>45</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C39" s="2">
         <v>3.0</v>
@@ -1053,7 +1053,7 @@
         <v>46</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C40" s="2">
         <v>3.0</v>
@@ -1064,7 +1064,7 @@
         <v>47</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C41" s="2">
         <v>3.0</v>
@@ -1075,7 +1075,7 @@
         <v>48</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C42" s="2">
         <v>3.0</v>
@@ -1086,7 +1086,7 @@
         <v>49</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C43" s="2">
         <v>3.0</v>
@@ -1097,7 +1097,7 @@
         <v>50</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C44" s="2">
         <v>3.0</v>
@@ -1108,7 +1108,7 @@
         <v>51</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C45" s="2">
         <v>3.0</v>
@@ -1130,7 +1130,7 @@
         <v>53</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C47" s="2">
         <v>3.0</v>
@@ -1262,7 +1262,7 @@
         <v>65</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C59" s="2">
         <v>4.0</v>
@@ -1273,7 +1273,7 @@
         <v>66</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="C60" s="2">
         <v>4.0</v>
@@ -1281,10 +1281,10 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>68</v>
+        <v>7</v>
       </c>
       <c r="C61" s="2">
         <v>4.0</v>
@@ -1295,7 +1295,7 @@
         <v>69</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>4</v>
+        <v>67</v>
       </c>
       <c r="C62" s="2">
         <v>4.0</v>
@@ -1317,7 +1317,7 @@
         <v>71</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C64" s="2">
         <v>4.0</v>
@@ -1328,7 +1328,7 @@
         <v>72</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C65" s="2">
         <v>4.0</v>
@@ -1364,8 +1364,8 @@
       <c r="B2" s="5">
         <v>16.0</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>74</v>
+      <c r="C2" s="5">
+        <v>20.5</v>
       </c>
     </row>
     <row r="3">
@@ -1373,10 +1373,10 @@
         <v>9</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
+      </c>
+      <c r="C3" s="5">
+        <v>7.5</v>
       </c>
     </row>
     <row r="4">
@@ -1384,10 +1384,10 @@
         <v>18</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
+      </c>
+      <c r="C4" s="5">
+        <v>7.5</v>
       </c>
     </row>
     <row r="5">
@@ -1395,10 +1395,10 @@
         <v>26</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
+      </c>
+      <c r="C5" s="5">
+        <v>12.5</v>
       </c>
     </row>
     <row r="6">
@@ -1406,53 +1406,65 @@
         <v>7</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
+      </c>
+      <c r="C6" s="5">
+        <v>13.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
+      </c>
+      <c r="C7" s="5">
+        <v>2.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>85</v>
+        <v>82</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="13">
@@ -1460,16 +1472,18 @@
         <v>71</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>88</v>
-      </c>
+      <c r="A14" s="6"/>
+      <c r="B14" s="9"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>